<commit_message>
style: Change product card aspect ratio from 3/4 to full and image to square
</commit_message>
<xml_diff>
--- a/홈페이지상품등록(HP72).xlsx
+++ b/홈페이지상품등록(HP72).xlsx
@@ -235,11 +235,11 @@
     <t>215/55R18</t>
   </si>
   <si>
-    <t>SUV/RV용</t>
+    <t>SUV용,사계절용,프리미엄,저소음,승차감</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>SUV/RV용,사계절용,프리미엄,저소음,승차감</t>
+    <t>SUV용</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -516,12 +516,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -539,6 +533,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -884,8 +884,8 @@
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
       <c r="E1" s="14"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="18"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="24"/>
       <c r="H1" s="6"/>
       <c r="I1" s="7"/>
       <c r="J1" s="12"/>
@@ -894,7 +894,7 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="17" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="15" t="s">
@@ -923,17 +923,17 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A3" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="22" t="s">
+      <c r="A3" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3" s="21">
         <v>471900</v>
       </c>
       <c r="D3" s="5">
-        <v>240669</v>
+        <v>275000</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
@@ -943,27 +943,27 @@
         <v>4</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A4" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="22" t="s">
+      <c r="A4" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="21">
         <v>482900</v>
       </c>
       <c r="D4" s="5">
-        <v>246279</v>
+        <v>281000</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
@@ -973,27 +973,27 @@
         <v>4</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="22" t="s">
+      <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="21">
         <v>467500</v>
       </c>
       <c r="D5" s="5">
-        <v>238425</v>
+        <v>273000</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
@@ -1003,27 +1003,27 @@
         <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A6" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="22" t="s">
+      <c r="A6" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="21">
         <v>488400</v>
       </c>
       <c r="D6" s="5">
-        <v>249084</v>
+        <v>284000</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
@@ -1033,27 +1033,27 @@
         <v>4</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A7" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="22" t="s">
+      <c r="A7" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="21">
         <v>423500</v>
       </c>
       <c r="D7" s="5">
-        <v>215985</v>
+        <v>250000</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
@@ -1063,27 +1063,27 @@
         <v>4</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A8" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="22" t="s">
+      <c r="A8" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="21">
         <v>444400</v>
       </c>
       <c r="D8" s="5">
-        <v>226644</v>
+        <v>261000</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
@@ -1093,27 +1093,27 @@
         <v>4</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A9" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="22" t="s">
+      <c r="A9" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="21">
         <v>464200</v>
       </c>
       <c r="D9" s="5">
-        <v>236742</v>
+        <v>271000</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
@@ -1123,27 +1123,27 @@
         <v>4</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A10" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="22" t="s">
+      <c r="A10" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="21">
         <v>424600</v>
       </c>
       <c r="D10" s="5">
-        <v>216546</v>
+        <v>250000</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
@@ -1153,27 +1153,27 @@
         <v>4</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A11" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="22" t="s">
+      <c r="A11" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="21">
         <v>453200</v>
       </c>
       <c r="D11" s="5">
-        <v>231132</v>
+        <v>265000</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5" t="s">
@@ -1183,27 +1183,27 @@
         <v>4</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="21">
         <v>375100</v>
       </c>
       <c r="D12" s="5">
-        <v>191301</v>
+        <v>224000</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
@@ -1213,27 +1213,27 @@
         <v>4</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A13" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="22" t="s">
+      <c r="A13" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="21">
         <v>462000</v>
       </c>
       <c r="D13" s="5">
-        <v>235620</v>
+        <v>270000</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
@@ -1243,27 +1243,27 @@
         <v>4</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A14" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="22" t="s">
+      <c r="A14" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="21">
         <v>424600</v>
       </c>
       <c r="D14" s="5">
-        <v>216546</v>
+        <v>250000</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
@@ -1273,27 +1273,27 @@
         <v>4</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A15" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="22" t="s">
+      <c r="A15" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="21">
         <v>436700</v>
       </c>
       <c r="D15" s="5">
-        <v>222717</v>
+        <v>257000</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
@@ -1303,27 +1303,27 @@
         <v>4</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A16" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="22" t="s">
+      <c r="A16" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="21">
         <v>399300</v>
       </c>
       <c r="D16" s="5">
-        <v>203643</v>
+        <v>217000</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
@@ -1333,27 +1333,27 @@
         <v>4</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A17" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="22" t="s">
+      <c r="A17" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="21">
         <v>380600</v>
       </c>
       <c r="D17" s="5">
-        <v>194106</v>
+        <v>207000</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
@@ -1363,27 +1363,27 @@
         <v>4</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="21">
         <v>367400</v>
       </c>
       <c r="D18" s="5">
-        <v>187374</v>
+        <v>200000</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
@@ -1393,27 +1393,27 @@
         <v>4</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A19" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="22" t="s">
+      <c r="A19" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="21">
         <v>382800</v>
       </c>
       <c r="D19" s="5">
-        <v>195228</v>
+        <v>208000</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
@@ -1423,27 +1423,27 @@
         <v>4</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A20" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="22" t="s">
+      <c r="A20" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="21">
         <v>366300</v>
       </c>
       <c r="D20" s="5">
-        <v>186813</v>
+        <v>199000</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
@@ -1453,27 +1453,27 @@
         <v>4</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A21" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="22" t="s">
+      <c r="A21" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="21">
         <v>356400</v>
       </c>
       <c r="D21" s="5">
-        <v>181764</v>
+        <v>194000</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
@@ -1483,27 +1483,27 @@
         <v>4</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A22" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="22" t="s">
+      <c r="A22" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="21">
         <v>337700</v>
       </c>
       <c r="D22" s="5">
-        <v>172227</v>
+        <v>184000</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
@@ -1513,27 +1513,27 @@
         <v>4</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="22" t="s">
+      <c r="A23" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="21">
         <v>349800</v>
       </c>
       <c r="D23" s="5">
-        <v>178398</v>
+        <v>190000</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
@@ -1543,27 +1543,27 @@
         <v>4</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A24" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="22" t="s">
+      <c r="A24" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="21">
         <v>360800</v>
       </c>
       <c r="D24" s="5">
-        <v>184008</v>
+        <v>196000</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
@@ -1573,27 +1573,27 @@
         <v>4</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A25" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" s="22" t="s">
+      <c r="A25" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="21">
         <v>404800</v>
       </c>
       <c r="D25" s="5">
-        <v>206448</v>
+        <v>220000</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="5" t="s">
@@ -1603,27 +1603,27 @@
         <v>4</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A26" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" s="22" t="s">
+      <c r="A26" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="21">
         <v>385000</v>
       </c>
       <c r="D26" s="5">
-        <v>196350</v>
+        <v>209000</v>
       </c>
       <c r="E26" s="5"/>
       <c r="F26" s="5" t="s">
@@ -1633,27 +1633,27 @@
         <v>4</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A27" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B27" s="22" t="s">
+      <c r="A27" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="21">
         <v>364100</v>
       </c>
       <c r="D27" s="5">
-        <v>185691</v>
+        <v>198000</v>
       </c>
       <c r="E27" s="5"/>
       <c r="F27" s="5" t="s">
@@ -1663,29 +1663,29 @@
         <v>4</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A28" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="22" t="s">
+      <c r="A28" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="21">
         <v>343200</v>
       </c>
       <c r="D28" s="5">
-        <v>175032</v>
-      </c>
-      <c r="E28" s="24"/>
+        <v>187000</v>
+      </c>
+      <c r="E28" s="22"/>
       <c r="F28" s="5" t="s">
         <v>4</v>
       </c>
@@ -1693,29 +1693,29 @@
         <v>4</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="50.1" customHeight="1">
-      <c r="A29" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B29" s="22" t="s">
+      <c r="A29" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="21">
         <v>328900</v>
       </c>
       <c r="D29" s="5">
-        <v>167739</v>
-      </c>
-      <c r="E29" s="24"/>
+        <v>179000</v>
+      </c>
+      <c r="E29" s="22"/>
       <c r="F29" s="5" t="s">
         <v>4</v>
       </c>
@@ -1723,27 +1723,27 @@
         <v>4</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="16.5">
-      <c r="A30" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B30" s="22" t="s">
+      <c r="A30" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="21">
         <v>324500</v>
       </c>
       <c r="D30" s="9">
-        <v>165495</v>
+        <v>177000</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>4</v>
@@ -1752,27 +1752,27 @@
         <v>4</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16.5">
-      <c r="A31" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B31" s="22" t="s">
+      <c r="A31" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="21">
         <v>288200</v>
       </c>
       <c r="D31" s="9">
-        <v>146982</v>
+        <v>157000</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>4</v>
@@ -1781,27 +1781,27 @@
         <v>4</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16.5">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="23">
+      <c r="C32" s="21">
         <v>346500</v>
       </c>
       <c r="D32" s="9">
-        <v>176715</v>
+        <v>189000</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>4</v>
@@ -1810,27 +1810,27 @@
         <v>4</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="16.5">
-      <c r="A33" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B33" s="22" t="s">
+      <c r="A33" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="21">
         <v>297000</v>
       </c>
       <c r="D33" s="9">
-        <v>151470</v>
+        <v>162000</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>4</v>
@@ -1839,27 +1839,27 @@
         <v>4</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="16.5">
-      <c r="A34" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="22" t="s">
+      <c r="A34" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="23">
+      <c r="C34" s="21">
         <v>279400</v>
       </c>
       <c r="D34" s="9">
-        <v>142494</v>
+        <v>153000</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>4</v>
@@ -1868,27 +1868,27 @@
         <v>4</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="16.5">
-      <c r="A35" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B35" s="22" t="s">
+      <c r="A35" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="23">
+      <c r="C35" s="21">
         <v>319000</v>
       </c>
       <c r="D35" s="9">
-        <v>162690</v>
+        <v>174000</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>4</v>
@@ -1897,27 +1897,27 @@
         <v>4</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="16.5">
-      <c r="A36" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B36" s="22" t="s">
+      <c r="A36" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="23">
+      <c r="C36" s="21">
         <v>293700</v>
       </c>
       <c r="D36" s="9">
-        <v>149787</v>
+        <v>160000</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>4</v>
@@ -1926,27 +1926,27 @@
         <v>4</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J36" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="16.5">
-      <c r="A37" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B37" s="22" t="s">
+      <c r="A37" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="23">
+      <c r="C37" s="21">
         <v>323400</v>
       </c>
       <c r="D37" s="9">
-        <v>164934</v>
+        <v>176000</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>4</v>
@@ -1955,27 +1955,27 @@
         <v>4</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="16.5">
-      <c r="A38" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="23">
+      <c r="C38" s="21">
         <v>301400</v>
       </c>
       <c r="D38" s="9">
-        <v>153714</v>
+        <v>164000</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>4</v>
@@ -1984,27 +1984,27 @@
         <v>4</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="16.5">
-      <c r="A39" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="22" t="s">
+      <c r="A39" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C39" s="23">
+      <c r="C39" s="21">
         <v>275000</v>
       </c>
       <c r="D39" s="9">
-        <v>140250</v>
+        <v>150000</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>4</v>
@@ -2013,27 +2013,27 @@
         <v>4</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="16.5">
-      <c r="A40" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B40" s="22" t="s">
+      <c r="A40" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C40" s="23">
+      <c r="C40" s="21">
         <v>259600</v>
       </c>
       <c r="D40" s="9">
-        <v>132396</v>
+        <v>142000</v>
       </c>
       <c r="F40" s="5" t="s">
         <v>4</v>
@@ -2042,27 +2042,27 @@
         <v>4</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16.5">
-      <c r="A41" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="22" t="s">
+      <c r="A41" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="23">
+      <c r="C41" s="21">
         <v>249700</v>
       </c>
       <c r="D41" s="9">
-        <v>127347</v>
+        <v>137000</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>4</v>
@@ -2071,27 +2071,27 @@
         <v>4</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="16.5">
-      <c r="A42" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B42" s="22" t="s">
+      <c r="A42" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="23">
+      <c r="C42" s="21">
         <v>259600</v>
       </c>
       <c r="D42" s="9">
-        <v>132396</v>
+        <v>142000</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>4</v>
@@ -2100,27 +2100,27 @@
         <v>4</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="16.5">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C43" s="23">
+      <c r="C43" s="21">
         <v>265100</v>
       </c>
       <c r="D43" s="9">
-        <v>135201</v>
+        <v>145000</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>4</v>
@@ -2129,27 +2129,27 @@
         <v>4</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J43" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="16.5">
-      <c r="A44" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B44" s="22" t="s">
+      <c r="A44" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C44" s="23">
+      <c r="C44" s="21">
         <v>248600</v>
       </c>
       <c r="D44" s="9">
-        <v>126786</v>
+        <v>136000</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>4</v>
@@ -2158,27 +2158,27 @@
         <v>4</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16.5">
-      <c r="A45" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B45" s="22" t="s">
+      <c r="A45" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C45" s="23">
+      <c r="C45" s="21">
         <v>239800</v>
       </c>
       <c r="D45" s="9">
-        <v>122298</v>
+        <v>131000</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>4</v>
@@ -2187,27 +2187,27 @@
         <v>4</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="16.5">
-      <c r="A46" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B46" s="22" t="s">
+      <c r="A46" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C46" s="23">
+      <c r="C46" s="21">
         <v>251900</v>
       </c>
       <c r="D46" s="9">
-        <v>128469</v>
+        <v>138000</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>4</v>
@@ -2216,27 +2216,27 @@
         <v>4</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="16.5">
-      <c r="A47" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B47" s="22" t="s">
+      <c r="A47" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="23">
+      <c r="C47" s="21">
         <v>305800</v>
       </c>
       <c r="D47" s="9">
-        <v>155958</v>
+        <v>167000</v>
       </c>
       <c r="F47" s="5" t="s">
         <v>4</v>
@@ -2245,27 +2245,27 @@
         <v>4</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="16.5">
-      <c r="A48" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="22" t="s">
+      <c r="A48" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C48" s="23">
+      <c r="C48" s="21">
         <v>294800</v>
       </c>
       <c r="D48" s="9">
-        <v>150348</v>
+        <v>161000</v>
       </c>
       <c r="F48" s="5" t="s">
         <v>4</v>
@@ -2274,27 +2274,27 @@
         <v>4</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16.5">
-      <c r="A49" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" s="22" t="s">
+      <c r="A49" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C49" s="23">
+      <c r="C49" s="21">
         <v>233200</v>
       </c>
       <c r="D49" s="9">
-        <v>118932</v>
+        <v>128000</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>4</v>
@@ -2303,27 +2303,27 @@
         <v>4</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J49" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="16.5">
-      <c r="A50" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B50" s="22" t="s">
+      <c r="A50" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C50" s="23">
+      <c r="C50" s="21">
         <v>278300</v>
       </c>
       <c r="D50" s="9">
-        <v>141933</v>
+        <v>152000</v>
       </c>
       <c r="F50" s="5" t="s">
         <v>4</v>
@@ -2332,27 +2332,27 @@
         <v>4</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J50" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="16.5">
-      <c r="A51" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B51" s="22" t="s">
+      <c r="A51" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="23">
+      <c r="C51" s="21">
         <v>254100</v>
       </c>
       <c r="D51" s="9">
-        <v>129591</v>
+        <v>139000</v>
       </c>
       <c r="F51" s="5" t="s">
         <v>4</v>
@@ -2361,27 +2361,27 @@
         <v>4</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J51" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="16.5">
-      <c r="A52" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B52" s="22" t="s">
+      <c r="A52" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C52" s="23">
+      <c r="C52" s="21">
         <v>213400</v>
       </c>
       <c r="D52" s="9">
-        <v>108834</v>
+        <v>117000</v>
       </c>
       <c r="F52" s="5" t="s">
         <v>4</v>
@@ -2390,27 +2390,27 @@
         <v>4</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J52" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="16.5">
-      <c r="A53" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" s="22" t="s">
+      <c r="A53" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C53" s="23">
+      <c r="C53" s="21">
         <v>253000</v>
       </c>
       <c r="D53" s="9">
-        <v>129030</v>
+        <v>138000</v>
       </c>
       <c r="F53" s="5" t="s">
         <v>4</v>
@@ -2419,27 +2419,27 @@
         <v>4</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J53" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="16.5">
-      <c r="A54" s="21" t="s">
+      <c r="A54" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C54" s="23">
+      <c r="C54" s="21">
         <v>200200</v>
       </c>
       <c r="D54" s="9">
-        <v>102102</v>
+        <v>110000</v>
       </c>
       <c r="F54" s="5" t="s">
         <v>4</v>
@@ -2448,27 +2448,27 @@
         <v>4</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J54" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="16.5">
-      <c r="A55" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" s="22" t="s">
+      <c r="A55" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C55" s="23">
+      <c r="C55" s="21">
         <v>192500</v>
       </c>
       <c r="D55" s="9">
-        <v>98175</v>
+        <v>106000</v>
       </c>
       <c r="F55" s="5" t="s">
         <v>4</v>
@@ -2477,13 +2477,13 @@
         <v>4</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J55" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>